<commit_message>
fix: resolve Sprint 1 P0 issues #6, #7, #8, #9
- #6: Prevent negative stock — decrementStock() now validates
  available >= requested before decrementing, throws StateError if not
- #7: Add PIN rate limiting — lock account for 5 min after 5 failed
  attempts on login and unlock flows
- #8: Add error handling to syncFromDb() — differentiate auth, parse,
  and network errors; log via debugPrint; return error message to caller
- #9: Fix batch decrement silent success — throw StateError when
  batchId is provided but not found, instead of silently falling through

Updated backlog tracker to mark #6, #7, #8, #9 as Fixed.

https://claude.ai/code/session_01YZM8C6T9r1Rx28goApvBWQ
</commit_message>
<xml_diff>
--- a/BillReady_2.0_Prioritized_Backlog.xlsx
+++ b/BillReady_2.0_Prioritized_Backlog.xlsx
@@ -971,7 +971,7 @@
       </c>
       <c r="K7" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="K8" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1077,7 @@
       </c>
       <c r="K9" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
       </c>
       <c r="K10" s="24" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve Sprint 2 issues #11, #12, #13, #18, #19, #21, #22
- #11: Add GST rounding to 2 decimal places (nearest paisa) across all
  GstCalculator methods to prevent floating-point accumulation errors
- #12: Add cgst/sgst/igst fields to ReturnLineItem and SalesReturn for
  GSTR-1 filing compliance on returns
- #13: Validate return qty <= original bill qty in addReturn(), accounting
  for previously returned quantities
- #18: Extract _resetActiveState() in BillProvider, eliminating 4
  duplicated 12-field reset blocks
- #19: Add global error handlers (FlutterError.onError and
  PlatformDispatcher.onError) in main() to catch unhandled errors
- #21: Fix ReportService month iteration bug where month 12+1=13 could
  overflow in _buildMonthlyPnL()
- #22: Add exponential backoff retry (3 attempts, 1s/2s/4s) to
  DbService _upsert() and _selectAll() for transient network failures

Updated backlog tracker to mark all 7 issues as Fixed.

https://claude.ai/code/session_01YZM8C6T9r1Rx28goApvBWQ
</commit_message>
<xml_diff>
--- a/BillReady_2.0_Prioritized_Backlog.xlsx
+++ b/BillReady_2.0_Prioritized_Backlog.xlsx
@@ -1236,7 +1236,7 @@
       </c>
       <c r="K12" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="K13" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
       </c>
       <c r="K14" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1607,7 +1607,7 @@
       </c>
       <c r="K19" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="K20" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1766,7 @@
       </c>
       <c r="K22" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1819,7 @@
       </c>
       <c r="K23" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add serial number management to DbService and implement tests
- Introduced methods for saving and retrieving serial numbers in DbService.
- Added new test files for bill total footer, create bill workflow, payment screen, product list screen, and cross-provider E2E tests to ensure functionality and integration.
- Enhanced existing tests to cover new features and maintain code quality.

This update supports better inventory tracking and management for products.
</commit_message>
<xml_diff>
--- a/BillReady_2.0_Prioritized_Backlog.xlsx
+++ b/BillReady_2.0_Prioritized_Backlog.xlsx
@@ -1990,7 +1990,7 @@
       </c>
       <c r="K26" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="K27" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="K28" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
       </c>
       <c r="K29" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="K30" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="K31" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="K32" s="26" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="K33" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="K36" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="K37" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="K38" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="K39" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="K40" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>N/A - crypto is used for PIN hashing</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="K41" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="K42" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -2997,7 +2997,7 @@
       </c>
       <c r="K45" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3050,7 +3050,7 @@
       </c>
       <c r="K46" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="K47" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="K48" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3209,7 +3209,7 @@
       </c>
       <c r="K49" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3262,7 +3262,7 @@
       </c>
       <c r="K50" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="K53" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="K54" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="K55" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
       </c>
       <c r="K56" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3633,7 +3633,7 @@
       </c>
       <c r="K57" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3686,7 +3686,7 @@
       </c>
       <c r="K58" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3739,7 +3739,7 @@
       </c>
       <c r="K59" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="K60" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3845,7 +3845,7 @@
       </c>
       <c r="K61" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3898,7 +3898,7 @@
       </c>
       <c r="K62" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="K63" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4004,7 +4004,7 @@
       </c>
       <c r="K64" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="K65" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="K66" s="30" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
     </row>

</xml_diff>